<commit_message>
EKSTalks og MUSE har fået status tester for afsendelse af Shared EKD Recording og XDS Metadata.
</commit_message>
<xml_diff>
--- a/html/EOJ-Systemer_excel.XLSX
+++ b/html/EOJ-Systemer_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5EA485-C29D-466C-871D-9CF737EBACBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C77E83C-546E-4861-BB65-09DB80D1096D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
     <t>Sensum Bosted _EOJ_ (EG)</t>
   </si>
   <si>
-    <t>VITAE Suite (Dedalus)</t>
+    <t>VITAE Suite (Dedalus Healthcare Denmark)</t>
   </si>
   <si>
     <t>Acknowledgement</t>

</xml_diff>